<commit_message>
sudah bisa import ralan dan ranap
</commit_message>
<xml_diff>
--- a/public/templates/template-import-tarif-ralan.xlsx
+++ b/public/templates/template-import-tarif-ralan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\smc-internal-app\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B67E62D5-C10A-44C4-B62E-C8F5494CDB96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42EF6F8-B79D-435D-AA29-576E8FD199A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{E1829FB7-46DE-47B0-B1A0-4B6669D1A06F}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>kd_jenis_prw</t>
   </si>
@@ -73,9 +73,6 @@
   </si>
   <si>
     <t>AKTE KELAHIRAN</t>
-  </si>
-  <si>
-    <t>Administrasi</t>
   </si>
   <si>
     <t>-</t>
@@ -114,9 +111,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -437,107 +433,106 @@
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>100000</v>
       </c>
-      <c r="E2" s="2">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2">
-        <v>0</v>
-      </c>
-      <c r="G2" s="2">
-        <v>0</v>
-      </c>
-      <c r="H2" s="2">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0</v>
-      </c>
-      <c r="J2" s="2">
-        <v>0</v>
-      </c>
-      <c r="K2" s="2">
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
         <v>100000</v>
       </c>
-      <c r="L2" s="2">
-        <v>0</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>17</v>
+      <c r="L2" s="1">
+        <v>0</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>